<commit_message>
Updated the worksheet name to "How to complete a manifest"
</commit_message>
<xml_diff>
--- a/edp_schema_template_v0.1.xlsx
+++ b/edp_schema_template_v0.1.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zef22hak/development/COPO_refactoring/COPO-production/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-production/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24EEECBE-4C71-2742-8E08-8D4A3D161A5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB344638-AF08-7041-A1ED-1783CFDAFA15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{964001A8-9378-804A-8584-54773ECBCFFA}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18060" xr2:uid="{964001A8-9378-804A-8584-54773ECBCFFA}"/>
   </bookViews>
   <sheets>
-    <sheet name="How to complete the Manifest" sheetId="3" r:id="rId1"/>
+    <sheet name="How to complete the manifest" sheetId="3" r:id="rId1"/>
     <sheet name="sample" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -260,10 +260,10 @@
     <t>For the use of Earlham Institute only - DO NOT EDIT</t>
   </si>
   <si>
-    <t>Instructions for completing the Manifest.</t>
+    <t>Do not edit fields highlighted in grey, these are for Earlham Institute use only</t>
   </si>
   <si>
-    <t>Do not edit fields highlighted in grey, these are for Earlham Institute use only</t>
+    <t>Instructions for completing the manifest.</t>
   </si>
 </sst>
 </file>
@@ -682,130 +682,67 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -833,6 +770,69 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1177,7 +1177,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" ht="21" x14ac:dyDescent="0.2">
       <c r="A1" s="19" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" s="20"/>
     </row>
@@ -1187,7 +1187,7 @@
     </row>
     <row r="3" spans="1:2" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" s="24"/>
     </row>
@@ -1205,13 +1205,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="26" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="68"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="48"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -1247,11 +1247,11 @@
       <c r="R2" s="1"/>
     </row>
     <row r="3" spans="1:18" ht="21" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="70"/>
-      <c r="C3" s="71"/>
+      <c r="B3" s="50"/>
+      <c r="C3" s="51"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -1269,12 +1269,12 @@
       <c r="R3" s="1"/>
     </row>
     <row r="4" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="75"/>
+      <c r="B4" s="53"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="55"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -1285,20 +1285,20 @@
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
-      <c r="O4" s="76" t="s">
+      <c r="O4" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="P4" s="73"/>
-      <c r="Q4" s="71"/>
+      <c r="P4" s="53"/>
+      <c r="Q4" s="51"/>
       <c r="R4" s="1"/>
     </row>
     <row r="5" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="72" t="s">
+      <c r="A5" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="73"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="77"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="57"/>
       <c r="E5" s="6" t="s">
         <v>5</v>
       </c>
@@ -1311,28 +1311,28 @@
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
-      <c r="O5" s="78" t="s">
+      <c r="O5" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="P5" s="79"/>
-      <c r="Q5" s="80"/>
+      <c r="P5" s="59"/>
+      <c r="Q5" s="60"/>
       <c r="R5" s="1"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="35"/>
-      <c r="I6" s="35"/>
-      <c r="J6" s="35"/>
-      <c r="K6" s="31"/>
-      <c r="L6" s="36"/>
+      <c r="B6" s="67"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="70"/>
+      <c r="F6" s="71"/>
+      <c r="G6" s="71"/>
+      <c r="H6" s="71"/>
+      <c r="I6" s="71"/>
+      <c r="J6" s="71"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="72"/>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="2"/>
@@ -1341,18 +1341,18 @@
       <c r="R6" s="1"/>
     </row>
     <row r="7" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="32"/>
-      <c r="B7" s="33"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="38"/>
-      <c r="G7" s="38"/>
-      <c r="H7" s="38"/>
-      <c r="I7" s="38"/>
-      <c r="J7" s="38"/>
-      <c r="K7" s="39"/>
-      <c r="L7" s="40"/>
+      <c r="A7" s="68"/>
+      <c r="B7" s="69"/>
+      <c r="C7" s="69"/>
+      <c r="D7" s="69"/>
+      <c r="E7" s="73"/>
+      <c r="F7" s="74"/>
+      <c r="G7" s="74"/>
+      <c r="H7" s="74"/>
+      <c r="I7" s="74"/>
+      <c r="J7" s="74"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="45"/>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
@@ -1361,19 +1361,19 @@
       <c r="R7" s="7"/>
     </row>
     <row r="8" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39"/>
-      <c r="I8" s="39"/>
-      <c r="J8" s="39"/>
-      <c r="K8" s="40"/>
+      <c r="B8" s="76"/>
+      <c r="C8" s="76"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="45"/>
       <c r="L8" s="8"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
@@ -1383,20 +1383,20 @@
       <c r="R8" s="1"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A9" s="43" t="s">
+      <c r="A9" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="44"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="44"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="44"/>
-      <c r="J9" s="44"/>
-      <c r="K9" s="45"/>
-      <c r="L9" s="52"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="27"/>
+      <c r="L9" s="78"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
@@ -1405,18 +1405,18 @@
       <c r="R9" s="1"/>
     </row>
     <row r="10" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="46"/>
-      <c r="B10" s="47"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
-      <c r="J10" s="47"/>
-      <c r="K10" s="48"/>
-      <c r="L10" s="53"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="79"/>
       <c r="M10" s="9"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
@@ -1425,103 +1425,103 @@
       <c r="R10" s="1"/>
     </row>
     <row r="11" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="49"/>
-      <c r="B11" s="50"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="50"/>
-      <c r="J11" s="50"/>
-      <c r="K11" s="51"/>
-      <c r="L11" s="54"/>
+      <c r="A11" s="31"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="33"/>
+      <c r="L11" s="80"/>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
-      <c r="O11" s="55" t="s">
+      <c r="O11" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="P11" s="44"/>
-      <c r="Q11" s="44"/>
-      <c r="R11" s="45"/>
+      <c r="P11" s="26"/>
+      <c r="Q11" s="26"/>
+      <c r="R11" s="27"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A12" s="56" t="s">
+      <c r="A12" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="57"/>
-      <c r="C12" s="57"/>
-      <c r="D12" s="57"/>
-      <c r="E12" s="57"/>
-      <c r="F12" s="57"/>
-      <c r="G12" s="57"/>
-      <c r="H12" s="57"/>
-      <c r="I12" s="57"/>
-      <c r="J12" s="57"/>
-      <c r="K12" s="58"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="35"/>
+      <c r="H12" s="35"/>
+      <c r="I12" s="35"/>
+      <c r="J12" s="35"/>
+      <c r="K12" s="36"/>
       <c r="L12" s="10"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
-      <c r="O12" s="46"/>
-      <c r="P12" s="47"/>
-      <c r="Q12" s="47"/>
-      <c r="R12" s="48"/>
+      <c r="O12" s="28"/>
+      <c r="P12" s="29"/>
+      <c r="Q12" s="29"/>
+      <c r="R12" s="30"/>
     </row>
     <row r="13" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="59"/>
-      <c r="B13" s="60"/>
-      <c r="C13" s="60"/>
-      <c r="D13" s="60"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="60"/>
-      <c r="H13" s="60"/>
-      <c r="I13" s="60"/>
-      <c r="J13" s="60"/>
-      <c r="K13" s="61"/>
+      <c r="A13" s="37"/>
+      <c r="B13" s="38"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
+      <c r="J13" s="38"/>
+      <c r="K13" s="39"/>
       <c r="L13" s="11"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
-      <c r="O13" s="49"/>
-      <c r="P13" s="50"/>
-      <c r="Q13" s="50"/>
-      <c r="R13" s="51"/>
+      <c r="O13" s="31"/>
+      <c r="P13" s="32"/>
+      <c r="Q13" s="32"/>
+      <c r="R13" s="33"/>
     </row>
     <row r="14" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="59"/>
-      <c r="B14" s="60"/>
-      <c r="C14" s="60"/>
-      <c r="D14" s="60"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="60"/>
-      <c r="G14" s="60"/>
-      <c r="H14" s="60"/>
-      <c r="I14" s="60"/>
-      <c r="J14" s="60"/>
-      <c r="K14" s="61"/>
+      <c r="A14" s="37"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="38"/>
+      <c r="J14" s="38"/>
+      <c r="K14" s="39"/>
       <c r="L14" s="11"/>
       <c r="M14" s="12"/>
       <c r="N14" s="12"/>
-      <c r="O14" s="65" t="s">
+      <c r="O14" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="P14" s="39"/>
-      <c r="Q14" s="39"/>
-      <c r="R14" s="40"/>
+      <c r="P14" s="44"/>
+      <c r="Q14" s="44"/>
+      <c r="R14" s="45"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A15" s="59"/>
-      <c r="B15" s="60"/>
-      <c r="C15" s="60"/>
-      <c r="D15" s="60"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="60"/>
-      <c r="H15" s="60"/>
-      <c r="I15" s="60"/>
-      <c r="J15" s="60"/>
-      <c r="K15" s="61"/>
+      <c r="A15" s="37"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="38"/>
+      <c r="I15" s="38"/>
+      <c r="J15" s="38"/>
+      <c r="K15" s="39"/>
       <c r="L15" s="11"/>
       <c r="M15" s="12"/>
       <c r="N15" s="12"/>
@@ -1531,17 +1531,17 @@
       <c r="R15" s="1"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A16" s="59"/>
-      <c r="B16" s="60"/>
-      <c r="C16" s="60"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
-      <c r="G16" s="60"/>
-      <c r="H16" s="60"/>
-      <c r="I16" s="60"/>
-      <c r="J16" s="60"/>
-      <c r="K16" s="61"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="38"/>
+      <c r="J16" s="38"/>
+      <c r="K16" s="39"/>
       <c r="L16" s="11"/>
       <c r="M16" s="12"/>
       <c r="N16" s="12"/>
@@ -1551,17 +1551,17 @@
       <c r="R16" s="1"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A17" s="59"/>
-      <c r="B17" s="60"/>
-      <c r="C17" s="60"/>
-      <c r="D17" s="60"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="60"/>
-      <c r="H17" s="60"/>
-      <c r="I17" s="60"/>
-      <c r="J17" s="60"/>
-      <c r="K17" s="61"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="38"/>
+      <c r="J17" s="38"/>
+      <c r="K17" s="39"/>
       <c r="L17" s="11"/>
       <c r="M17" s="12"/>
       <c r="N17" s="12"/>
@@ -1571,17 +1571,17 @@
       <c r="R17" s="1"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A18" s="59"/>
-      <c r="B18" s="60"/>
-      <c r="C18" s="60"/>
-      <c r="D18" s="60"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="60"/>
-      <c r="G18" s="60"/>
-      <c r="H18" s="60"/>
-      <c r="I18" s="60"/>
-      <c r="J18" s="60"/>
-      <c r="K18" s="61"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="38"/>
+      <c r="I18" s="38"/>
+      <c r="J18" s="38"/>
+      <c r="K18" s="39"/>
       <c r="L18" s="11"/>
       <c r="M18" s="12"/>
       <c r="N18" s="12"/>
@@ -1591,17 +1591,17 @@
       <c r="R18" s="1"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A19" s="59"/>
-      <c r="B19" s="60"/>
-      <c r="C19" s="60"/>
-      <c r="D19" s="60"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="60"/>
-      <c r="G19" s="60"/>
-      <c r="H19" s="60"/>
-      <c r="I19" s="60"/>
-      <c r="J19" s="60"/>
-      <c r="K19" s="61"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="38"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="38"/>
+      <c r="I19" s="38"/>
+      <c r="J19" s="38"/>
+      <c r="K19" s="39"/>
       <c r="L19" s="11"/>
       <c r="M19" s="12"/>
       <c r="N19" s="12"/>
@@ -1611,17 +1611,17 @@
       <c r="R19" s="1"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A20" s="59"/>
-      <c r="B20" s="60"/>
-      <c r="C20" s="60"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="60"/>
-      <c r="H20" s="60"/>
-      <c r="I20" s="60"/>
-      <c r="J20" s="60"/>
-      <c r="K20" s="61"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="38"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="38"/>
+      <c r="H20" s="38"/>
+      <c r="I20" s="38"/>
+      <c r="J20" s="38"/>
+      <c r="K20" s="39"/>
       <c r="L20" s="11"/>
       <c r="M20" s="12"/>
       <c r="N20" s="12"/>
@@ -1631,17 +1631,17 @@
       <c r="R20" s="1"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A21" s="59"/>
-      <c r="B21" s="60"/>
-      <c r="C21" s="60"/>
-      <c r="D21" s="60"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="60"/>
-      <c r="H21" s="60"/>
-      <c r="I21" s="60"/>
-      <c r="J21" s="60"/>
-      <c r="K21" s="61"/>
+      <c r="A21" s="37"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="38"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="38"/>
+      <c r="J21" s="38"/>
+      <c r="K21" s="39"/>
       <c r="L21" s="11"/>
       <c r="M21" s="12"/>
       <c r="N21" s="12"/>
@@ -1651,17 +1651,17 @@
       <c r="R21" s="1"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A22" s="59"/>
-      <c r="B22" s="60"/>
-      <c r="C22" s="60"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="60"/>
-      <c r="H22" s="60"/>
-      <c r="I22" s="60"/>
-      <c r="J22" s="60"/>
-      <c r="K22" s="61"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="38"/>
+      <c r="I22" s="38"/>
+      <c r="J22" s="38"/>
+      <c r="K22" s="39"/>
       <c r="L22" s="11"/>
       <c r="M22" s="12"/>
       <c r="N22" s="12"/>
@@ -1671,17 +1671,17 @@
       <c r="R22" s="1"/>
     </row>
     <row r="23" spans="1:18" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="62"/>
-      <c r="B23" s="63"/>
-      <c r="C23" s="63"/>
-      <c r="D23" s="63"/>
-      <c r="E23" s="63"/>
-      <c r="F23" s="63"/>
-      <c r="G23" s="63"/>
-      <c r="H23" s="63"/>
-      <c r="I23" s="63"/>
-      <c r="J23" s="63"/>
-      <c r="K23" s="64"/>
+      <c r="A23" s="40"/>
+      <c r="B23" s="41"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="41"/>
+      <c r="H23" s="41"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="41"/>
+      <c r="K23" s="42"/>
       <c r="L23" s="11"/>
       <c r="M23" s="12"/>
       <c r="N23" s="12"/>
@@ -1731,11 +1731,11 @@
       <c r="R25" s="1"/>
     </row>
     <row r="26" spans="1:18" ht="20" x14ac:dyDescent="0.2">
-      <c r="A26" s="25" t="s">
+      <c r="A26" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="26"/>
-      <c r="C26" s="27"/>
+      <c r="B26" s="62"/>
+      <c r="C26" s="63"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -1753,13 +1753,13 @@
       <c r="R26" s="13"/>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
+      <c r="B27" s="65"/>
+      <c r="C27" s="65"/>
+      <c r="D27" s="65"/>
+      <c r="E27" s="65"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
@@ -1776,6 +1776,13 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A6:D7"/>
+    <mergeCell ref="E6:L7"/>
+    <mergeCell ref="A8:K8"/>
+    <mergeCell ref="A9:K11"/>
+    <mergeCell ref="L9:L11"/>
     <mergeCell ref="O11:R13"/>
     <mergeCell ref="A12:K23"/>
     <mergeCell ref="O14:R14"/>
@@ -1787,13 +1794,6 @@
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A6:D7"/>
-    <mergeCell ref="E6:L7"/>
-    <mergeCell ref="A8:K8"/>
-    <mergeCell ref="A9:K11"/>
-    <mergeCell ref="L9:L11"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Please select" sqref="L8" xr:uid="{5295E0F2-B1D8-1D4A-9C6B-C01C8ABCA05C}">

</xml_diff>